<commit_message>
feat: frontend et configs complets
</commit_message>
<xml_diff>
--- a/backend/templates/BOM 1.xlsx
+++ b/backend/templates/BOM 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30021"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NH445\Documents\Cimelta\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\docgen-platform\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD637DF5-0522-4DDA-807F-25888F4D5690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAA7EB2D-9A93-4F35-A02F-E38307B8E0C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" xr2:uid="{A5E7338C-5E6E-4A4C-9DF5-37B1037E6A05}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t>#</t>
   </si>
@@ -42,12 +42,6 @@
     <t>Qty</t>
   </si>
   <si>
-    <t>GPL</t>
-  </si>
-  <si>
-    <t>Discount final</t>
-  </si>
-  <si>
     <t>Unit Price</t>
   </si>
   <si>
@@ -63,9 +57,6 @@
     <t>Aruba 6200F 24G PoE+ (R8N87A)</t>
   </si>
   <si>
-    <t>CIMELTA</t>
-  </si>
-  <si>
     <t>1.2</t>
   </si>
   <si>
@@ -133,6 +124,9 @@
   </si>
   <si>
     <t>Samsung 55" BET-H Series 4K Business TV BE55T-H</t>
+  </si>
+  <si>
+    <t>Client : CIMELTA</t>
   </si>
 </sst>
 </file>
@@ -460,9 +454,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="17">
+  <cellStyleXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -479,14 +472,11 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -505,9 +495,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="166" fontId="3" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -523,18 +510,15 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="2" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -572,24 +556,23 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="17">
-    <cellStyle name="Comma 2" xfId="3" xr:uid="{D69DC2DF-CD03-43E1-B231-BDE27095C328}"/>
-    <cellStyle name="Comma 2 2" xfId="15" xr:uid="{9BE0EA1C-DE90-4C77-952A-CDDE9501C124}"/>
-    <cellStyle name="Currency 2" xfId="4" xr:uid="{2AEB43E3-811D-40A4-803E-FC5D4778D2EB}"/>
-    <cellStyle name="Currency 2 2" xfId="5" xr:uid="{F029817C-35D3-4BB0-A18B-04A02A8B4AE7}"/>
-    <cellStyle name="Currency 3" xfId="6" xr:uid="{31FA19DB-9858-432F-9F23-34FE4BAAC18B}"/>
-    <cellStyle name="Monétaire 2" xfId="7" xr:uid="{462CF98A-0DC6-498D-A6D0-08A8A53F3669}"/>
+  <cellStyles count="16">
+    <cellStyle name="Comma 2" xfId="2" xr:uid="{D69DC2DF-CD03-43E1-B231-BDE27095C328}"/>
+    <cellStyle name="Comma 2 2" xfId="14" xr:uid="{9BE0EA1C-DE90-4C77-952A-CDDE9501C124}"/>
+    <cellStyle name="Currency 2" xfId="3" xr:uid="{2AEB43E3-811D-40A4-803E-FC5D4778D2EB}"/>
+    <cellStyle name="Currency 2 2" xfId="4" xr:uid="{F029817C-35D3-4BB0-A18B-04A02A8B4AE7}"/>
+    <cellStyle name="Currency 3" xfId="5" xr:uid="{31FA19DB-9858-432F-9F23-34FE4BAAC18B}"/>
+    <cellStyle name="Monétaire 2" xfId="6" xr:uid="{462CF98A-0DC6-498D-A6D0-08A8A53F3669}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="8" xr:uid="{25AF97B0-F3BF-44D4-A381-A9082710E5A6}"/>
-    <cellStyle name="Normal 2 2" xfId="9" xr:uid="{9BD6C37A-2A1D-4410-A995-A2302D424D89}"/>
-    <cellStyle name="Normal 2 6" xfId="10" xr:uid="{AF356917-3510-4FC7-9FB0-B4492ABE3DBB}"/>
-    <cellStyle name="Normal 3" xfId="11" xr:uid="{D6340309-A40B-4BC6-B582-9F721EA7399B}"/>
-    <cellStyle name="Normal 3 2" xfId="12" xr:uid="{029DFDA3-AECB-445B-A5FB-4857725C7A99}"/>
-    <cellStyle name="Normal 4" xfId="13" xr:uid="{C304AA9C-4784-4264-B381-3A7F8C5B6222}"/>
-    <cellStyle name="Normal 5" xfId="2" xr:uid="{9A8DAA5D-AEFC-468F-B12F-F89FDAA92D9E}"/>
-    <cellStyle name="Normal 5 2" xfId="16" xr:uid="{5F00FAC1-FDD7-4DC6-84ED-8262E0C5E6BD}"/>
-    <cellStyle name="Normal 6" xfId="14" xr:uid="{068FC2A2-6A5C-4CB2-9234-551EEDBDB117}"/>
-    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
+    <cellStyle name="Normal 2" xfId="7" xr:uid="{25AF97B0-F3BF-44D4-A381-A9082710E5A6}"/>
+    <cellStyle name="Normal 2 2" xfId="8" xr:uid="{9BD6C37A-2A1D-4410-A995-A2302D424D89}"/>
+    <cellStyle name="Normal 2 6" xfId="9" xr:uid="{AF356917-3510-4FC7-9FB0-B4492ABE3DBB}"/>
+    <cellStyle name="Normal 3" xfId="10" xr:uid="{D6340309-A40B-4BC6-B582-9F721EA7399B}"/>
+    <cellStyle name="Normal 3 2" xfId="11" xr:uid="{029DFDA3-AECB-445B-A5FB-4857725C7A99}"/>
+    <cellStyle name="Normal 4" xfId="12" xr:uid="{C304AA9C-4784-4264-B381-3A7F8C5B6222}"/>
+    <cellStyle name="Normal 5" xfId="1" xr:uid="{9A8DAA5D-AEFC-468F-B12F-F89FDAA92D9E}"/>
+    <cellStyle name="Normal 5 2" xfId="15" xr:uid="{5F00FAC1-FDD7-4DC6-84ED-8262E0C5E6BD}"/>
+    <cellStyle name="Normal 6" xfId="13" xr:uid="{068FC2A2-6A5C-4CB2-9234-551EEDBDB117}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -901,27 +884,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BABFDAF0-E923-43C4-A174-28EA523A1C73}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="16.09765625" customWidth="1"/>
     <col min="7" max="7" width="23.296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="23"/>
-      <c r="D1" s="24" t="s">
+      <c r="C1" s="20"/>
+      <c r="D1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
       <c r="H1" s="1" t="s">
         <v>3</v>
       </c>
@@ -931,316 +914,272 @@
       <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="24"/>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="23"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="B4" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="14"/>
+      <c r="D4" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I4" s="6">
+        <v>22</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="D5" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="6">
+        <v>18</v>
+      </c>
+      <c r="J5" s="7">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="D6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="6">
+        <v>4</v>
+      </c>
+      <c r="J6" s="7">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="D7" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I7" s="6">
+        <v>2</v>
+      </c>
+      <c r="J7" s="7">
+        <v>0</v>
+      </c>
+      <c r="K7" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="D8" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I8" s="6">
+        <v>2</v>
+      </c>
+      <c r="J8" s="7">
+        <v>0</v>
+      </c>
+      <c r="K8" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="26"/>
+      <c r="D9" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="I9" s="11">
         <v>8</v>
       </c>
+      <c r="J9" s="12">
+        <v>0</v>
+      </c>
+      <c r="K9" s="12">
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="27"/>
+    <row r="10" spans="1:11" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="D10" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I10" s="6">
+        <v>1</v>
+      </c>
+      <c r="J10" s="7">
+        <v>0</v>
+      </c>
+      <c r="K10" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
-        <v>1</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="6"/>
+    <row r="11" spans="1:11" ht="35.299999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="D11" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="I11" s="6">
+        <v>2</v>
+      </c>
+      <c r="J11" s="7">
+        <v>0</v>
+      </c>
+      <c r="K11" s="7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="17"/>
-      <c r="F4" s="17"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I4" s="7">
-        <v>22</v>
-      </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="9">
-        <v>0</v>
-      </c>
-      <c r="L4" s="8">
-        <v>0</v>
-      </c>
-      <c r="M4" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="18"/>
-      <c r="D5" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I5" s="7">
-        <v>18</v>
-      </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="9">
-        <v>0</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0</v>
-      </c>
-      <c r="M5" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I6" s="7">
-        <v>4</v>
-      </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="9">
-        <v>0</v>
-      </c>
-      <c r="L6" s="8">
-        <v>0</v>
-      </c>
-      <c r="M6" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="18"/>
-      <c r="D7" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I7" s="7">
-        <v>2</v>
-      </c>
-      <c r="J7" s="8"/>
-      <c r="K7" s="9">
-        <v>0</v>
-      </c>
-      <c r="L7" s="8">
-        <v>0</v>
-      </c>
-      <c r="M7" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I8" s="7">
-        <v>2</v>
-      </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="9">
-        <v>0</v>
-      </c>
-      <c r="L8" s="8">
-        <v>0</v>
-      </c>
-      <c r="M8" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B9" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="28" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="I9" s="13">
+    <row r="12" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="J9" s="14"/>
-      <c r="K9" s="15">
-        <v>0</v>
-      </c>
-      <c r="L9" s="14">
-        <v>0</v>
-      </c>
-      <c r="M9" s="14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="35.299999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="16" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I10" s="7">
-        <v>1</v>
-      </c>
-      <c r="J10" s="8"/>
-      <c r="K10" s="9">
-        <v>0</v>
-      </c>
-      <c r="L10" s="8">
-        <v>0</v>
-      </c>
-      <c r="M10" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="35.299999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="I11" s="7">
-        <v>2</v>
-      </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="9">
-        <v>0</v>
-      </c>
-      <c r="L11" s="8">
-        <v>0</v>
-      </c>
-      <c r="M11" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
-      <c r="J12" s="20"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="21"/>
-      <c r="M12" s="10">
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="18"/>
+      <c r="K12" s="8">
         <v>0</v>
       </c>
     </row>
@@ -1249,16 +1188,10 @@
     <row r="24" ht="30.85" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:G8"/>
-    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A12:J12"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:G1"/>
-    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D4:G4"/>
@@ -1270,6 +1203,12 @@
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="D11:G11"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:G8"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>